<commit_message>
Generated 300 mock test cases each for Selenium, Appium, Vulnerability, and Load tests along with Excel reports
</commit_message>
<xml_diff>
--- a/Vulnerability Test Results/dependency-report.xlsx
+++ b/Vulnerability Test Results/dependency-report.xlsx
@@ -546,7 +546,7 @@
     <row r="1" ht="32" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>DentAI — Dependency &amp; Supply Chain Report</t>
+          <t>DentAI â€” Dependency &amp; Supply Chain Report</t>
         </is>
       </c>
     </row>
@@ -1183,7 +1183,7 @@
       </c>
       <c r="H17" s="6" t="inlineStr">
         <is>
-          <t>Correct use — keep</t>
+          <t>Correct use â€” keep</t>
         </is>
       </c>
     </row>
@@ -1389,7 +1389,7 @@
     <row r="1" ht="32" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>DentAI — Performance &amp; Load Test Results</t>
+          <t>DentAI â€” Performance &amp; Load Test Results</t>
         </is>
       </c>
     </row>
@@ -1496,7 +1496,7 @@
       </c>
       <c r="K4" s="4" t="inlineStr">
         <is>
-          <t>New DB conn per request — main bottleneck</t>
+          <t>New DB conn per request â€” main bottleneck</t>
         </is>
       </c>
     </row>
@@ -1582,7 +1582,7 @@
       </c>
       <c r="K6" s="4" t="inlineStr">
         <is>
-          <t>Failure point approaching — pool exhausted</t>
+          <t>Failure point approaching â€” pool exhausted</t>
         </is>
       </c>
     </row>
@@ -1632,7 +1632,7 @@
     <row r="8" ht="22" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>Spike (50→500)</t>
+          <t>Spike (50â†’500)</t>
         </is>
       </c>
       <c r="B8" s="4" t="n">
@@ -1797,7 +1797,7 @@
       </c>
       <c r="K11" s="6" t="inlineStr">
         <is>
-          <t>Slight degradation — connection pressure</t>
+          <t>Slight degradation â€” connection pressure</t>
         </is>
       </c>
     </row>
@@ -1883,7 +1883,7 @@
       </c>
       <c r="K13" s="6" t="inlineStr">
         <is>
-          <t>Significant degradation — potential memory leak</t>
+          <t>Significant degradation â€” potential memory leak</t>
         </is>
       </c>
     </row>
@@ -1926,7 +1926,7 @@
       </c>
       <c r="K14" s="4" t="inlineStr">
         <is>
-          <t>No DB dependency — fast baseline</t>
+          <t>No DB dependency â€” fast baseline</t>
         </is>
       </c>
     </row>
@@ -2002,7 +2002,7 @@
     <row r="1" ht="32" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>DentAI — Secrets &amp; Credential Scan Results</t>
+          <t>DentAI â€” Secrets &amp; Credential Scan Results</t>
         </is>
       </c>
     </row>
@@ -2073,7 +2073,7 @@
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>Remove immediately — use .env</t>
+          <t>Remove immediately â€” use .env</t>
         </is>
       </c>
     </row>
@@ -2105,7 +2105,7 @@
       </c>
       <c r="F5" s="6" t="inlineStr">
         <is>
-          <t>Remove immediately — use .env</t>
+          <t>Remove immediately â€” use .env</t>
         </is>
       </c>
     </row>
@@ -2137,7 +2137,7 @@
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>Remove immediately — use .env</t>
+          <t>Remove immediately â€” use .env</t>
         </is>
       </c>
     </row>
@@ -2169,7 +2169,7 @@
       </c>
       <c r="F7" s="6" t="inlineStr">
         <is>
-          <t>Remove immediately — use .env</t>
+          <t>Remove immediately â€” use .env</t>
         </is>
       </c>
     </row>

</xml_diff>